<commit_message>
Refresh Main cap table to Q2'26 / Aug'26
Price, shares outstanding, cash, debt, and accumulated deficit were all
Q3'24 vintage. Updated from SLS's Q2'26 10-Q (SEC EDGAR sls-20260630.htm)
and 9/11/26 closing price; dated source comments added on each input cell.
Share count is ~2.9x the old figure (warrant dilution), so EV moves from
~$1.0B to ~$2.2B. MC/EV formulas untouched.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SLS.xlsx
+++ b/SLS.xlsx
@@ -23,7 +23,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Arial"/>
       <family val="2"/>
@@ -51,6 +51,11 @@
       <color theme="1"/>
       <sz val="10"/>
       <u val="single"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="000000FF"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="3">
@@ -166,7 +171,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -232,6 +237,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="4" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -312,6 +319,52 @@
 </file>
 
 <file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Claude</author>
+  </authors>
+  <commentList>
+    <comment ref="L2" authorId="0" shapeId="0">
+      <text>
+        <t>Updated 9/11/26. SLS closing price 9/11/26 = $11.55, down 14.4% on the day (from ~$13.49) on elevated volume with NO new company filing or disclosed trial result behind the move -- read as pre-catalyst de-risking, not readout news. Two binary catalysts (REGAL OS + SLS009 front-line topline) both guided for Q4 2026. Re-pull live price before sizing anything off this cell; it has moved &gt;10% intraday twice in the past three weeks.
+Source: stockanalysis.com/stocks/sls (close 9/11/26); corroborated by MarketBeat/StockTitan same-day coverage of the 14.4% drop.</t>
+      </text>
+    </comment>
+    <comment ref="L3" authorId="0" shapeId="0">
+      <text>
+        <t>Was 70.381979 (Q3'24) -- ~2.9x dilution since, mostly warrant exercises and the 2026 ATM authorization (unused as of this filing).
+Source: SLS 10-Q for Q2'26, cover page: "As of August 10, 2026, SELLAS Life Sciences Group, Inc. had outstanding 201,945,709 shares of common stock." SEC EDGAR: sec.gov/Archives/edgar/data/0001390478/000139047826000012/sls-20260630.htm
+(Balance-sheet-date count as of 6/30/26 was 201,918,874 -- essentially identical; cover-page count used here as the more current figure.)</t>
+      </text>
+    </comment>
+    <comment ref="L5" authorId="0" shapeId="0">
+      <text>
+        <t>Was 21.031 (Q3'24).
+Source: SLS 10-Q for Q2'26, balance sheet, cash and cash equivalents as of 6/30/26 = $138.3M. Confirmed in Q2'26 earnings release (GlobeNewswire, 8/11/26). Note H1'26 net cash used in operating activities was $16.4M (see REGAL Failure Floor tab) -- the cash balance rose q/q anyway on warrant-exercise proceeds, so don't infer burn rate from the raw cash delta.</t>
+      </text>
+    </comment>
+    <comment ref="L6" authorId="0" shapeId="0">
+      <text>
+        <t>Was =4.547+5.49 (Q3'24). Company carries no funded debt; the two components here are operating lease liabilities (NY HQ) as of 6/30/26: current $0.580M + non-current $0.157M = $0.737M total.
+Source: SLS 10-Q for Q2'26 balance sheet, SEC EDGAR (sls-20260630.htm).</t>
+      </text>
+    </comment>
+    <comment ref="L9" authorId="0" shapeId="0">
+      <text>
+        <t>NOT re-verified in this pass (was 237.188 as of Q3'24). Doesn't feed MC/EV so left as-is; pull current additional paid-in capital from the Q2'26 10-Q balance sheet before relying on it.</t>
+      </text>
+    </comment>
+    <comment ref="L10" authorId="0" shapeId="0">
+      <text>
+        <t>Was -234.28 (Q3'24).
+Source: SLS 10-Q for Q2'26 balance sheet: accumulated deficit of $293.0M as of 6/30/26. SEC EDGAR (sls-20260630.htm).</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment2.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>tc={3F632F91-120B-4288-A788-6998CFC973C8}</author>
@@ -900,8 +953,8 @@
           <t>Price</t>
         </is>
       </c>
-      <c r="L2" s="21" t="n">
-        <v>14.45</v>
+      <c r="L2" s="33" t="n">
+        <v>11.55</v>
       </c>
     </row>
     <row r="3">
@@ -930,12 +983,12 @@
           <t>Shares</t>
         </is>
       </c>
-      <c r="L3" s="1" t="n">
-        <v>70.381979</v>
+      <c r="L3" s="34" t="n">
+        <v>201.945709</v>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>Q324</t>
+          <t>8/10/26</t>
         </is>
       </c>
     </row>
@@ -976,12 +1029,12 @@
           <t>Cash</t>
         </is>
       </c>
-      <c r="L5" s="1" t="n">
-        <v>21.031</v>
+      <c r="L5" s="34" t="n">
+        <v>138.3</v>
       </c>
       <c r="M5" s="2" t="inlineStr">
         <is>
-          <t>Q324</t>
+          <t>6/30/26</t>
         </is>
       </c>
     </row>
@@ -999,13 +1052,13 @@
           <t>Debt</t>
         </is>
       </c>
-      <c r="L6" s="1">
-        <f>4.547+5.49</f>
+      <c r="L6" s="34">
+        <f>0.580+0.157</f>
         <v/>
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t>Q324</t>
+          <t>6/30/26</t>
         </is>
       </c>
     </row>
@@ -1044,8 +1097,8 @@
           <t>AD</t>
         </is>
       </c>
-      <c r="L10" s="1" t="n">
-        <v>-234.28</v>
+      <c r="L10" s="34" t="n">
+        <v>-293</v>
       </c>
     </row>
     <row r="12">
@@ -1065,6 +1118,7 @@
     <hyperlink ref="B3" location="'galinpepimut-S'!A1" display="galinpepimut-S"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Add REGAL Failure Floor tab with SLS009 scenario levers
Per-share SOTP floor conditional on GPS failing: net cash at readout
(sourced burn rate from Q2'26 10-Q operating cash flow) plus a low/mid/high
SLS009 risk-adjusted value lever ($30M/$100M/$200M) plus a GPS-residual
input (default $0). Outputs implied floor $/share and downside from spot
per scenario. Notes the panic-overshoot caveat and flags the unconfirmed
third-party report of REGAL's 80th event.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SLS.xlsx
+++ b/SLS.xlsx
@@ -14,6 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Patients" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="18mo Scenario" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="24mo Scenario" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="REGAL Failure Floor" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -22,8 +23,15 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="5">
+  <numFmts count="6">
+    <numFmt numFmtId="164" formatCode="$#,##0.0"/>
+    <numFmt numFmtId="165" formatCode="#,##0.0"/>
+    <numFmt numFmtId="166" formatCode="$#,##0.00"/>
+    <numFmt numFmtId="167" formatCode="0.0"/>
+    <numFmt numFmtId="168" formatCode="$#,##0"/>
+    <numFmt numFmtId="169" formatCode="0.0%"/>
+  </numFmts>
+  <fonts count="10">
     <font>
       <name val="Arial"/>
       <family val="2"/>
@@ -57,8 +65,32 @@
       <color rgb="000000FF"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00008000"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -69,6 +101,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFF0000"/>
         <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFF00"/>
+        <bgColor rgb="00FFFF00"/>
       </patternFill>
     </fill>
   </fills>
@@ -171,7 +209,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -239,6 +277,26 @@
     </xf>
     <xf numFmtId="4" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="4" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="4" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -376,6 +434,36 @@
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
     60 discontinuations</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment3.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Claude</author>
+  </authors>
+  <commentList>
+    <comment ref="C8" authorId="0" shapeId="0">
+      <text>
+        <t>Source: SLS 10-Q for Q2'26 (SEC EDGAR, sls-20260630.htm), condensed cash flow statement: net cash used in operating activities of $16.4M for the six months ended 6/30/26 (flat vs. H1'25), i.e. $16.4M / 2 quarters = $8.2M/quarter. As of 9/11/26.</t>
+      </text>
+    </comment>
+    <comment ref="C9" authorId="0" shapeId="0">
+      <text>
+        <t>2.0 quarters = burn from 7/1/26 through year-end 2026, matching the company's Q4'26 topline guidance. If the readout slips to Q1 2027 (real risk per the brief -- REGAL was still short of its confirmed 80th event as of 9/11/26), bump this to ~3.0 to add roughly one more quarter (~$8M) of burn. As of 9/11/26.</t>
+      </text>
+    </comment>
+    <comment ref="C12" authorId="0" shapeId="0">
+      <text>
+        <t>Default $0 per the bear case: GPS assumed worthless to equityholders on a REGAL miss. Could in principle reflect already-banked, non-refundable ex-China (3D Medicines) license economics, or optionality from a positive secondary/subgroup signal surviving a missed primary OS endpoint -- raise only with explicit justification, this is meant to stay conservative.</t>
+      </text>
+    </comment>
+    <comment ref="C16" authorId="0" shapeId="0">
+      <text>
+        <t>Illustrative risk-adjusted value levers for SLS009 (tambiciclib), not a formal rNPV build -- set by feel, refine as data emerges. Context: prior r/r AML Ph2 showed 46% ORR (29% CR/CRi), mOS 8.9mo in the least-pretreated cohort vs. ~2.5mo historical, no DLTs (ASH 2025); front-line randomized Ph2 (~80pts, response-rate endpoint, FDA-aligned, possible accelerated-approval path) had 28/80 enrolled with topline also guided for Q4 2026 per the Q2'26 update (SEC EDGAR, sls-20260630.htm / GlobeNewswire 8/11/26). Low/Mid/High = $30M/$100M/$200M per the brief's own bracketing; adjust as SLS009 data reads out.</t>
       </text>
     </comment>
   </commentList>
@@ -17784,4 +17872,248 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B1:E24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="2.8" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="B1" s="35" t="inlineStr">
+        <is>
+          <t>REGAL Failure Floor — Sum-of-the-Parts on GPS Failure</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="42" customHeight="1">
+      <c r="B2" s="36" t="inlineStr">
+        <is>
+          <t>Per-share value floor assuming REGAL misses and GPS is worth $0 to equityholders. This is the reference level for sizing / setting the strike on a defined-risk long-put position into the readout — it is NOT a price target, an expected value, or a prediction of the outcome. See Main and galinpepimut-S tabs for the full bear/bull case.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" s="37" t="inlineStr">
+        <is>
+          <t>Inputs</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="38" t="inlineStr">
+        <is>
+          <t>Current cash ($M)</t>
+        </is>
+      </c>
+      <c r="C5" s="39">
+        <f>Main!L5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="38" t="inlineStr">
+        <is>
+          <t>Current shares outstanding (M)</t>
+        </is>
+      </c>
+      <c r="C6" s="40">
+        <f>Main!L3</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="38" t="inlineStr">
+        <is>
+          <t>Current price ($, for reference)</t>
+        </is>
+      </c>
+      <c r="C7" s="41">
+        <f>Main!L2</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="38" t="inlineStr">
+        <is>
+          <t>Quarterly operating cash burn ($M)</t>
+        </is>
+      </c>
+      <c r="C8" s="42" t="n">
+        <v>8.199999999999999</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="38" t="inlineStr">
+        <is>
+          <t>Quarters of burn to readout</t>
+        </is>
+      </c>
+      <c r="C9" s="43" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="38" t="inlineStr">
+        <is>
+          <t>Est. burn to readout ($M)</t>
+        </is>
+      </c>
+      <c r="C10" s="44">
+        <f>C8*C9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="37" t="inlineStr">
+        <is>
+          <t>Net cash at readout ($M)</t>
+        </is>
+      </c>
+      <c r="C11" s="45">
+        <f>C5-C10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="38" t="inlineStr">
+        <is>
+          <t>GPS-residual / other value ($M)</t>
+        </is>
+      </c>
+      <c r="C12" s="46" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="37" t="inlineStr">
+        <is>
+          <t>SLS009 risk-adjusted value — scenario ($M)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="C15" s="47" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="D15" s="47" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="E15" s="47" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="38" t="inlineStr">
+        <is>
+          <t>SLS009 value ($M)</t>
+        </is>
+      </c>
+      <c r="C16" s="48" t="n">
+        <v>30</v>
+      </c>
+      <c r="D16" s="48" t="n">
+        <v>100</v>
+      </c>
+      <c r="E16" s="48" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="38" t="inlineStr">
+        <is>
+          <t>Implied floor value ($M)</t>
+        </is>
+      </c>
+      <c r="C18" s="44">
+        <f>$C$11+C16+$C$12</f>
+        <v/>
+      </c>
+      <c r="D18" s="44">
+        <f>$C$11+D16+$C$12</f>
+        <v/>
+      </c>
+      <c r="E18" s="44">
+        <f>$C$11+E16+$C$12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="37" t="inlineStr">
+        <is>
+          <t>Implied floor ($/share)</t>
+        </is>
+      </c>
+      <c r="C19" s="49">
+        <f>C18/$C$6</f>
+        <v/>
+      </c>
+      <c r="D19" s="49">
+        <f>D18/$C$6</f>
+        <v/>
+      </c>
+      <c r="E19" s="49">
+        <f>E18/$C$6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="38" t="inlineStr">
+        <is>
+          <t>Implied downside from current price</t>
+        </is>
+      </c>
+      <c r="C20" s="50">
+        <f>C19/$C$7-1</f>
+        <v/>
+      </c>
+      <c r="D20" s="50">
+        <f>D19/$C$7-1</f>
+        <v/>
+      </c>
+      <c r="E20" s="50">
+        <f>E19/$C$7-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22" ht="42" customHeight="1">
+      <c r="B22" s="36" t="inlineStr">
+        <is>
+          <t>A shocking/outright REGAL miss can gap the stock below this computed SOTP floor for hours to days before any mean-reversion -- treat this as a fundamental reference level for where to set a long-put strike, not a hard technical floor the price can't pierce intraday.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="56" customHeight="1">
+      <c r="B24" s="36" t="inlineStr">
+        <is>
+          <t>REGAL status as of 9/11/26: company-confirmed event count remains 78/80 (last reaffirmed via 3D Medicines disclosure 8/18/26). An unconfirmed third-party report (AktienCheck, ~8/23/26) claimed the 80th event had been reached; SELLAS has not issued a press release or filing confirming this, and stocktwits/retail reaction was skeptical. Re-check company IR / SEC EDGAR for an actual topline announcement before finalizing any position -- if confirmed, database lock/unblinding timelines could pull the readout forward of the Q4'26 guidance embedded above.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="B24:E24"/>
+    <mergeCell ref="B22:E22"/>
+    <mergeCell ref="B2:E2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+</worksheet>
 </file>
</xml_diff>